<commit_message>
Nuevas columnas para Lixis en pestaña de productos
</commit_message>
<xml_diff>
--- a/Formulario_Masterdata.xlsx
+++ b/Formulario_Masterdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollos\implementador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB23CE0-1C6A-4B4F-887A-C7E267A36F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6003291-F234-4261-AFC1-E63C3A25FED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" tabRatio="730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-900" windowWidth="29040" windowHeight="15840" tabRatio="730" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formulario de Registro" sheetId="2" r:id="rId1"/>
@@ -72,6 +72,44 @@
     <author>Gianpiero Tecca</author>
   </authors>
   <commentList>
+    <comment ref="F9" authorId="0" shapeId="0" xr:uid="{CCF1524E-367C-4191-BE32-7A8C06B22C36}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Solo si se envía a Lixis
+(opcional)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G9" authorId="0" shapeId="0" xr:uid="{069CE76A-1407-421C-AAB8-91FCF04DC864}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Solo si se envía a Lixis
+(opcional)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Gianpiero Tecca</author>
+  </authors>
+  <commentList>
     <comment ref="E9" authorId="0" shapeId="0" xr:uid="{70DC5BC4-43C0-478B-80E4-1A42D744F7D2}">
       <text>
         <r>
@@ -96,7 +134,7 @@
 </comments>
 </file>
 
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Gianpiero Tecca</author>
@@ -136,7 +174,7 @@
 </comments>
 </file>
 
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Gianpiero Tecca</author>
@@ -163,7 +201,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="241">
   <si>
     <t>GLN:</t>
   </si>
@@ -840,12 +878,6 @@
     <t>ONELITE</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>192.168.0.9</t>
   </si>
   <si>
@@ -870,46 +902,28 @@
     <t>Código Pallet:</t>
   </si>
   <si>
-    <t>00028273748473628192</t>
-  </si>
-  <si>
-    <t>00182728192837485912</t>
-  </si>
-  <si>
-    <t>00028273748473628193</t>
-  </si>
-  <si>
-    <t>00182728192837485911</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>12/10/2025</t>
-  </si>
-  <si>
-    <t>30-04-2026</t>
-  </si>
-  <si>
-    <t>2028-10-01</t>
-  </si>
-  <si>
-    <t>27364489102</t>
-  </si>
-  <si>
-    <t>27364489103</t>
-  </si>
-  <si>
-    <t>27364489104</t>
-  </si>
-  <si>
-    <t>27364489105</t>
+    <t>Capas por Pack:</t>
+  </si>
+  <si>
+    <t>Nivel de Agregación:</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>7790440527711</t>
+  </si>
+  <si>
+    <t>7795381000099</t>
+  </si>
+  <si>
+    <t>30503518599</t>
   </si>
 </sst>
 </file>
@@ -2000,11 +2014,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" style="20" bestFit="1" customWidth="1"/>
@@ -2012,38 +2026,48 @@
     <col min="3" max="3" width="21.85546875" style="20" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" style="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.42578125" style="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="15" style="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>16</v>
       </c>
@@ -2051,15 +2075,19 @@
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -2070,8 +2098,10 @@
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>24</v>
       </c>
@@ -2079,8 +2109,10 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
         <v>6</v>
       </c>
@@ -2096,8 +2128,14 @@
       <c r="E9" s="23" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" s="23" t="s">
+        <v>233</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>109</v>
       </c>
@@ -2111,8 +2149,12 @@
       <c r="E10" s="13" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="13"/>
+      <c r="G10" s="13" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>110</v>
       </c>
@@ -2122,8 +2164,10 @@
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>111</v>
       </c>
@@ -2139,8 +2183,10 @@
       <c r="E12" s="13" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
         <v>112</v>
       </c>
@@ -2150,8 +2196,12 @@
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
-    </row>
-    <row r="14" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F13" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>113</v>
       </c>
@@ -2161,8 +2211,10 @@
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
-    </row>
-    <row r="15" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+    </row>
+    <row r="15" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>114</v>
       </c>
@@ -2178,8 +2230,10 @@
       <c r="E15" s="13" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+    </row>
+    <row r="16" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
         <v>115</v>
       </c>
@@ -2189,8 +2243,12 @@
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
-    </row>
-    <row r="17" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F16" s="13"/>
+      <c r="G16" s="13" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
         <v>116</v>
       </c>
@@ -2206,8 +2264,10 @@
       <c r="E17" s="13" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>117</v>
       </c>
@@ -2217,8 +2277,12 @@
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
-    </row>
-    <row r="19" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="G18" s="13"/>
+    </row>
+    <row r="19" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
         <v>118</v>
       </c>
@@ -2232,291 +2296,386 @@
       <c r="E19" s="13" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>238</v>
+      </c>
       <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D20" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G20" s="13" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
       <c r="E27" s="13"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="13"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="13"/>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
       <c r="E29" s="13"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="13"/>
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
       <c r="E31" s="13"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
       <c r="E33" s="13"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F34" s="13"/>
+      <c r="G34" s="13"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
       <c r="E35" s="13"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F35" s="13"/>
+      <c r="G35" s="13"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="13"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="13"/>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
       <c r="E37" s="13"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F37" s="13"/>
+      <c r="G37" s="13"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="13"/>
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F38" s="13"/>
+      <c r="G38" s="13"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="13"/>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="13"/>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="13"/>
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
       <c r="D41" s="13"/>
       <c r="E41" s="13"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="13"/>
       <c r="B42" s="13"/>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="13"/>
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
       <c r="D43" s="13"/>
       <c r="E43" s="13"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="13"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="13"/>
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
       <c r="E45" s="13"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F45" s="13"/>
+      <c r="G45" s="13"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="13"/>
       <c r="B46" s="13"/>
       <c r="C46" s="13"/>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="13"/>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
       <c r="E47" s="13"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F47" s="13"/>
+      <c r="G47" s="13"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="13"/>
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F48" s="13"/>
+      <c r="G48" s="13"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="13"/>
       <c r="B49" s="13"/>
       <c r="C49" s="13"/>
       <c r="D49" s="13"/>
       <c r="E49" s="13"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13"/>
       <c r="B50" s="13"/>
       <c r="C50" s="13"/>
       <c r="D50" s="13"/>
       <c r="E50" s="13"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="13"/>
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
       <c r="D51" s="13"/>
       <c r="E51" s="13"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F51" s="13"/>
+      <c r="G51" s="13"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="13"/>
       <c r="B52" s="13"/>
       <c r="C52" s="13"/>
       <c r="D52" s="13"/>
       <c r="E52" s="13"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F52" s="13"/>
+      <c r="G52" s="13"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="13"/>
       <c r="B53" s="13"/>
       <c r="C53" s="13"/>
       <c r="D53" s="13"/>
       <c r="E53" s="13"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="13"/>
       <c r="B54" s="13"/>
       <c r="C54" s="13"/>
       <c r="D54" s="13"/>
       <c r="E54" s="13"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="13"/>
       <c r="B55" s="13"/>
       <c r="C55" s="13"/>
       <c r="D55" s="13"/>
       <c r="E55" s="13"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F55" s="13"/>
+      <c r="G55" s="13"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="13"/>
       <c r="B56" s="13"/>
       <c r="C56" s="13"/>
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="13"/>
       <c r="B57" s="13"/>
       <c r="C57" s="13"/>
       <c r="D57" s="13"/>
       <c r="E57" s="13"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="13"/>
       <c r="B58" s="13"/>
       <c r="C58" s="13"/>
       <c r="D58" s="13"/>
       <c r="E58" s="13"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="13"/>
       <c r="B59" s="13"/>
       <c r="C59" s="13"/>
       <c r="D59" s="13"/>
       <c r="E59" s="13"/>
+      <c r="F59" s="13"/>
+      <c r="G59" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="37" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -2760,11 +2919,21 @@
       </c>
     </row>
     <row r="19" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
+      <c r="A19" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="20" spans="1:5" s="14" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="13"/>
@@ -3542,7 +3711,7 @@
         <v>220</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>225</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -3556,7 +3725,7 @@
         <v>220</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>226</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -3567,10 +3736,10 @@
         <v>223</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -3650,7 +3819,7 @@
     </row>
     <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -3696,107 +3865,59 @@
         <v>96</v>
       </c>
       <c r="B9" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>229</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="E9" s="22" t="s">
         <v>231</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="F9" s="22" t="s">
         <v>232</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>233</v>
-      </c>
-      <c r="F9" s="22" t="s">
-        <v>234</v>
       </c>
       <c r="G9" s="22" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>236</v>
-      </c>
-      <c r="G10" s="21" t="s">
-        <v>93</v>
-      </c>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="21"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>243</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>237</v>
-      </c>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
       <c r="F11" s="13"/>
-      <c r="G11" s="21" t="s">
-        <v>108</v>
-      </c>
+      <c r="G11" s="21"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>244</v>
-      </c>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
       <c r="E12" s="13"/>
-      <c r="F12" s="13" t="s">
-        <v>238</v>
-      </c>
-      <c r="G12" s="21" t="s">
-        <v>108</v>
-      </c>
+      <c r="F12" s="13"/>
+      <c r="G12" s="21"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>242</v>
-      </c>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
-      <c r="G13" s="21" t="s">
-        <v>93</v>
-      </c>
+      <c r="G13" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -3809,6 +3930,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE275595-2AFF-44E8-A0B3-BEE1EB39E5E7}">
   <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C54"/>

</xml_diff>